<commit_message>
Function list v2: apply Confirmation Points answers of 19-Oct
- XD10 / XD09: case = destination x pcs/case (releases are multiples of
  pcs/case); unit stays whole; 1 case label = 1 case of 1 destination
- XD11: CONFLICT goods may go to another destination; PO qty not blocked;
  exception list = Log
- XD05 / XD01 / XD06 / XD07: parts that become Inactive are set No Sync and
  sent with CROSSDOCK_FLAG N; G-TOPAS without SFTP; SFTP / file / target
  tables not detailed
- Schedules: daily jobs after 27:30 with 3 retries; XD05 runs even if XD04
  failed; SERIAL_NO added by DB Surrounding; XD14 not used
- README / md decisions table; simulation text (any destination)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/function_list_v2/uiss/XD09_UISS_Batch_MappingCustomerOrderPO.xlsx
+++ b/deliverables/function_list_v2/uiss/XD09_UISS_Batch_MappingCustomerOrderPO.xlsx
@@ -32948,7 +32948,7 @@
       </c>
       <c r="BC9" s="948" t="inlineStr">
         <is>
-          <t>Unit = Part Number + Customer Order Date. Case = one per destination of the unit: the qty of</t>
+          <t>Unit = Part Number + Customer Order Date. Case = destination x pcs/case: the qty of a</t>
         </is>
       </c>
       <c r="BD9" s="941" t="n"/>
@@ -33057,7 +33057,7 @@
       <c r="BB10" s="941" t="n"/>
       <c r="BC10" s="948" t="inlineStr">
         <is>
-          <t>the destination is summed into one case (it never exceeds pcs/case).</t>
+          <t>destination is packed in cases of pcs/case (e.g. Vietnam 24 pcs, 6 pcs/case = 4 cases).</t>
         </is>
       </c>
       <c r="BD10" s="941" t="n"/>
@@ -33167,14 +33167,10 @@
       <c r="AY11" s="941" t="n"/>
       <c r="AZ11" s="943" t="n"/>
       <c r="BA11" s="941" t="n"/>
-      <c r="BB11" s="948" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="BB11" s="941" t="n"/>
       <c r="BC11" s="948" t="inlineStr">
         <is>
-          <t>Case Qty = number of destinations of the unit. PO Readiness (case) = cases whose whole qty</t>
+          <t>G-TOPAS releases in multiples of pcs/case (a remainder stays pending and is not in H0253), so</t>
         </is>
       </c>
       <c r="BD11" s="941" t="n"/>
@@ -33291,7 +33287,7 @@
       <c r="BB12" s="941" t="n"/>
       <c r="BC12" s="948" t="inlineStr">
         <is>
-          <t>is pre-mapped to a PO.</t>
+          <t>every case is full.</t>
         </is>
       </c>
       <c r="BD12" s="941" t="n"/>
@@ -33412,7 +33408,7 @@
       </c>
       <c r="BC13" s="948" t="inlineStr">
         <is>
-          <t>CROSSDOCK_STATUS '6' Ready: every line of the unit is pre-mapped. '7' Not Ready: at least</t>
+          <t>Case Qty = number of destinations of the unit. PO Readiness (case) = cases whose whole qty</t>
         </is>
       </c>
       <c r="BD13" s="941" t="n"/>
@@ -33525,7 +33521,7 @@
       <c r="BB14" s="941" t="n"/>
       <c r="BC14" s="948" t="inlineStr">
         <is>
-          <t>one line of the unit has no PO yet.</t>
+          <t>is pre-mapped to a PO.</t>
         </is>
       </c>
       <c r="BD14" s="941" t="n"/>
@@ -33646,7 +33642,7 @@
       </c>
       <c r="BC15" s="948" t="inlineStr">
         <is>
-          <t>Shown on XD10 as ASN Status Ready / Not Ready. Units with PO Readiness 0 are not listed</t>
+          <t>CROSSDOCK_STATUS '6' Ready: every line of the unit is pre-mapped. '7' Not Ready: at least</t>
         </is>
       </c>
       <c r="BD15" s="941" t="n"/>
@@ -33763,7 +33759,7 @@
       <c r="BB16" s="941" t="n"/>
       <c r="BC16" s="948" t="inlineStr">
         <is>
-          <t>on XD10; units already in a submitted ASN (ASN status '1' Created) are not taken</t>
+          <t>one line of the unit has no PO yet.</t>
         </is>
       </c>
       <c r="BD16" s="941" t="n"/>
@@ -33873,10 +33869,14 @@
       <c r="AY17" s="941" t="n"/>
       <c r="AZ17" s="943" t="n"/>
       <c r="BA17" s="941" t="n"/>
-      <c r="BB17" s="941" t="n"/>
+      <c r="BB17" s="948" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="BC17" s="948" t="inlineStr">
         <is>
-          <t>(PO_MAPPED_FLAG = 'Y').</t>
+          <t>Shown on XD10 as ASN Status Ready / Not Ready. Units with PO Readiness 0 are not listed</t>
         </is>
       </c>
       <c r="BD17" s="941" t="n"/>
@@ -33990,14 +33990,10 @@
       <c r="AY18" s="941" t="n"/>
       <c r="AZ18" s="943" t="n"/>
       <c r="BA18" s="941" t="n"/>
-      <c r="BB18" s="948" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="BB18" s="941" t="n"/>
       <c r="BC18" s="948" t="inlineStr">
         <is>
-          <t>The mapped qty is kept in the new table TB_R_PRA_DAILY_ORDER_MAPPED (no new</t>
+          <t>on XD10; units already in a submitted ASN (ASN status '1' Created) are not taken</t>
         </is>
       </c>
       <c r="BD18" s="941" t="n"/>
@@ -34106,7 +34102,7 @@
       <c r="BB19" s="941" t="n"/>
       <c r="BC19" s="948" t="inlineStr">
         <is>
-          <t>column in the Pra Daily Order); it is updated by [Create ASN] on XD10, not by this function.</t>
+          <t>(PO_MAPPED_FLAG = 'Y').</t>
         </is>
       </c>
       <c r="BD19" s="941" t="n"/>
@@ -34219,7 +34215,7 @@
       </c>
       <c r="BC20" s="948" t="inlineStr">
         <is>
-          <t>Nothing is saved by this function: #TEMP_INSTRUCTION is the pre-mapping only; the real</t>
+          <t>The mapped qty is kept in the new table TB_R_PRA_DAILY_ORDER_MAPPED (no new</t>
         </is>
       </c>
       <c r="BD20" s="941" t="n"/>
@@ -34328,7 +34324,7 @@
       <c r="BB21" s="941" t="n"/>
       <c r="BC21" s="948" t="inlineStr">
         <is>
-          <t>mapping is inserted into TB_R_INSTRUCTION by [Create ASN].</t>
+          <t>column in the Pra Daily Order); it is updated by [Create ASN] on XD10, not by this function.</t>
         </is>
       </c>
       <c r="BD21" s="941" t="n"/>
@@ -34434,8 +34430,16 @@
       <c r="AY22" s="941" t="n"/>
       <c r="AZ22" s="943" t="n"/>
       <c r="BA22" s="941" t="n"/>
-      <c r="BB22" s="941" t="n"/>
-      <c r="BC22" s="941" t="n"/>
+      <c r="BB22" s="948" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BC22" s="948" t="inlineStr">
+        <is>
+          <t>Nothing is saved by this function: #TEMP_INSTRUCTION is the pre-mapping only; the real</t>
+        </is>
+      </c>
       <c r="BD22" s="941" t="n"/>
       <c r="BE22" s="941" t="n"/>
       <c r="BF22" s="941" t="n"/>
@@ -34540,7 +34544,11 @@
       <c r="AZ23" s="943" t="n"/>
       <c r="BA23" s="941" t="n"/>
       <c r="BB23" s="941" t="n"/>
-      <c r="BC23" s="941" t="n"/>
+      <c r="BC23" s="948" t="inlineStr">
+        <is>
+          <t>mapping is inserted into TB_R_INSTRUCTION by [Create ASN].</t>
+        </is>
+      </c>
       <c r="BD23" s="941" t="n"/>
       <c r="BE23" s="941" t="n"/>
       <c r="BF23" s="941" t="n"/>

</xml_diff>

<commit_message>
UISS XD09/XD10: case may hold several COs and POs; new case screenshots
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QL8Do8Pd2rXEDNa1ifG2RK
</commit_message>
<xml_diff>
--- a/deliverables/function_list_v2/uiss/XD09_UISS_Batch_MappingCustomerOrderPO.xlsx
+++ b/deliverables/function_list_v2/uiss/XD09_UISS_Batch_MappingCustomerOrderPO.xlsx
@@ -33287,7 +33287,7 @@
       <c r="BB12" s="941" t="n"/>
       <c r="BC12" s="948" t="inlineStr">
         <is>
-          <t>every case is full.</t>
+          <t>every case is full. A case can hold several customer orders and several POs of the same</t>
         </is>
       </c>
       <c r="BD12" s="941" t="n"/>
@@ -33401,14 +33401,10 @@
       <c r="AY13" s="941" t="n"/>
       <c r="AZ13" s="943" t="n"/>
       <c r="BA13" s="941" t="n"/>
-      <c r="BB13" s="948" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="BB13" s="941" t="n"/>
       <c r="BC13" s="948" t="inlineStr">
         <is>
-          <t>Case Qty = number of destinations of the unit. PO Readiness (case) = cases whose whole qty</t>
+          <t>destination; a customer order line that does not fit in the remaining space of a case continues in</t>
         </is>
       </c>
       <c r="BD13" s="941" t="n"/>
@@ -33521,7 +33517,7 @@
       <c r="BB14" s="941" t="n"/>
       <c r="BC14" s="948" t="inlineStr">
         <is>
-          <t>is pre-mapped to a PO.</t>
+          <t>the next case (e.g. case 3 = CO-14001 4 + CO-14006 2 of PO2; case 4 = CO-14006 2 of PO2 +</t>
         </is>
       </c>
       <c r="BD14" s="941" t="n"/>
@@ -33635,14 +33631,10 @@
       <c r="AY15" s="941" t="n"/>
       <c r="AZ15" s="943" t="n"/>
       <c r="BA15" s="941" t="n"/>
-      <c r="BB15" s="948" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="BB15" s="941" t="n"/>
       <c r="BC15" s="948" t="inlineStr">
         <is>
-          <t>CROSSDOCK_STATUS '6' Ready: every line of the unit is pre-mapped. '7' Not Ready: at least</t>
+          <t>CO-14007 4 of PO4).</t>
         </is>
       </c>
       <c r="BD15" s="941" t="n"/>
@@ -33756,10 +33748,14 @@
       <c r="AY16" s="941" t="n"/>
       <c r="AZ16" s="943" t="n"/>
       <c r="BA16" s="941" t="n"/>
-      <c r="BB16" s="941" t="n"/>
+      <c r="BB16" s="948" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="BC16" s="948" t="inlineStr">
         <is>
-          <t>one line of the unit has no PO yet.</t>
+          <t>Case Qty = number of destinations of the unit. PO Readiness (case) = cases whose whole qty</t>
         </is>
       </c>
       <c r="BD16" s="941" t="n"/>
@@ -33869,14 +33865,10 @@
       <c r="AY17" s="941" t="n"/>
       <c r="AZ17" s="943" t="n"/>
       <c r="BA17" s="941" t="n"/>
-      <c r="BB17" s="948" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="BB17" s="941" t="n"/>
       <c r="BC17" s="948" t="inlineStr">
         <is>
-          <t>Shown on XD10 as ASN Status Ready / Not Ready. Units with PO Readiness 0 are not listed</t>
+          <t>is pre-mapped to a PO.</t>
         </is>
       </c>
       <c r="BD17" s="941" t="n"/>
@@ -33990,10 +33982,14 @@
       <c r="AY18" s="941" t="n"/>
       <c r="AZ18" s="943" t="n"/>
       <c r="BA18" s="941" t="n"/>
-      <c r="BB18" s="941" t="n"/>
+      <c r="BB18" s="948" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="BC18" s="948" t="inlineStr">
         <is>
-          <t>on XD10; units already in a submitted ASN (ASN status '1' Created) are not taken</t>
+          <t>CROSSDOCK_STATUS '6' Ready: every line of the unit is pre-mapped. '7' Not Ready: at least</t>
         </is>
       </c>
       <c r="BD18" s="941" t="n"/>
@@ -34102,7 +34098,7 @@
       <c r="BB19" s="941" t="n"/>
       <c r="BC19" s="948" t="inlineStr">
         <is>
-          <t>(PO_MAPPED_FLAG = 'Y').</t>
+          <t>one line of the unit has no PO yet.</t>
         </is>
       </c>
       <c r="BD19" s="941" t="n"/>
@@ -34215,7 +34211,7 @@
       </c>
       <c r="BC20" s="948" t="inlineStr">
         <is>
-          <t>The mapped qty is kept in the new table TB_R_PRA_DAILY_ORDER_MAPPED (no new</t>
+          <t>Shown on XD10 as ASN Status Ready / Not Ready. Units with PO Readiness 0 are not listed</t>
         </is>
       </c>
       <c r="BD20" s="941" t="n"/>
@@ -34324,7 +34320,7 @@
       <c r="BB21" s="941" t="n"/>
       <c r="BC21" s="948" t="inlineStr">
         <is>
-          <t>column in the Pra Daily Order); it is updated by [Create ASN] on XD10, not by this function.</t>
+          <t>on XD10; units already in a submitted ASN (ASN status '1' Created) are not taken</t>
         </is>
       </c>
       <c r="BD21" s="941" t="n"/>
@@ -34430,14 +34426,10 @@
       <c r="AY22" s="941" t="n"/>
       <c r="AZ22" s="943" t="n"/>
       <c r="BA22" s="941" t="n"/>
-      <c r="BB22" s="948" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="BB22" s="941" t="n"/>
       <c r="BC22" s="948" t="inlineStr">
         <is>
-          <t>Nothing is saved by this function: #TEMP_INSTRUCTION is the pre-mapping only; the real</t>
+          <t>(PO_MAPPED_FLAG = 'Y').</t>
         </is>
       </c>
       <c r="BD22" s="941" t="n"/>
@@ -34543,10 +34535,14 @@
       <c r="AY23" s="941" t="n"/>
       <c r="AZ23" s="943" t="n"/>
       <c r="BA23" s="941" t="n"/>
-      <c r="BB23" s="941" t="n"/>
+      <c r="BB23" s="948" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="BC23" s="948" t="inlineStr">
         <is>
-          <t>mapping is inserted into TB_R_INSTRUCTION by [Create ASN].</t>
+          <t>The mapped qty is kept in the new table TB_R_PRA_DAILY_ORDER_MAPPED (no new</t>
         </is>
       </c>
       <c r="BD23" s="941" t="n"/>
@@ -34653,7 +34649,11 @@
       <c r="AZ24" s="943" t="n"/>
       <c r="BA24" s="941" t="n"/>
       <c r="BB24" s="941" t="n"/>
-      <c r="BC24" s="941" t="n"/>
+      <c r="BC24" s="948" t="inlineStr">
+        <is>
+          <t>column in the Pra Daily Order); it is updated by [Create ASN] on XD10, not by this function.</t>
+        </is>
+      </c>
       <c r="BD24" s="941" t="n"/>
       <c r="BE24" s="941" t="n"/>
       <c r="BF24" s="941" t="n"/>
@@ -34757,8 +34757,16 @@
       <c r="AY25" s="941" t="n"/>
       <c r="AZ25" s="943" t="n"/>
       <c r="BA25" s="941" t="n"/>
-      <c r="BB25" s="941" t="n"/>
-      <c r="BC25" s="941" t="n"/>
+      <c r="BB25" s="948" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="BC25" s="948" t="inlineStr">
+        <is>
+          <t>Nothing is saved by this function: #TEMP_INSTRUCTION is the pre-mapping only; the real</t>
+        </is>
+      </c>
       <c r="BD25" s="941" t="n"/>
       <c r="BE25" s="941" t="n"/>
       <c r="BF25" s="941" t="n"/>
@@ -34863,7 +34871,11 @@
       <c r="AZ26" s="943" t="n"/>
       <c r="BA26" s="941" t="n"/>
       <c r="BB26" s="941" t="n"/>
-      <c r="BC26" s="941" t="n"/>
+      <c r="BC26" s="948" t="inlineStr">
+        <is>
+          <t>mapping is inserted into TB_R_INSTRUCTION by [Create ASN].</t>
+        </is>
+      </c>
       <c r="BD26" s="941" t="n"/>
       <c r="BE26" s="941" t="n"/>
       <c r="BF26" s="941" t="n"/>

</xml_diff>